<commit_message>
docs: record N-10 app refresh fallback progress
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,7 +1174,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09 background delivery code complete (Sep 15): observer queries for all nine metrics registered at launch, hourly background delivery enabled once a session exists, HealthKit acknowledged only after the batch is durably queued, single upload attempt per wake, concurrent wakes coalesced. Simulator build passes.</t>
+          <t>N-09 and N-10 code complete (Sep 15): observer queries for all nine metrics registered at launch with hourly background delivery, HealthKit acknowledged only after the batch is durably queued, single upload attempt per wake, concurrent wakes coalesced; BGAppRefreshTask fallback registered, chained and cancelled with the session. Simulator build passes.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15–21: N-09 background collection (code done Sep 15); N-10 BGTask fallback; N-11/N-14 notification + durable cold-start events; N-12 timer; N-13 one-per-day goal alerts; N-15 gong; N-16 Apple identity. Background delivery cannot be exercised on the simulator, so N-09 stays In progress until a signed device build is available.</t>
+          <t>Execution plan Sep 15–21: N-09 background collection (code done Sep 15); N-10 BGTask fallback (code done Sep 15); N-11/N-14 notification + durable cold-start events; N-12 timer; N-13 one-per-day goal alerts; N-15 gong; N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available.</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       <c r="G18" s="24" t="n"/>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I18" s="24" t="inlineStr">
@@ -2113,8 +2113,16 @@
           <t>Scheduled refresh runs when the observer does not fire</t>
         </is>
       </c>
-      <c r="J18" s="24" t="inlineStr"/>
-      <c r="K18" s="24" t="inlineStr"/>
+      <c r="J18" s="24" t="inlineStr">
+        <is>
+          <t>ios/Honoured/HealthBackgroundRefresh.swift, HonouredAppDelegate.swift, Info.plist · typecheck + simulator build Sep 15 · docs/bridge.md "Background sync"</t>
+        </is>
+      </c>
+      <c r="K18" s="24" t="inlineStr">
+        <is>
+          <t>Code complete. BGAppRefreshTask registered before launch finishes, rescheduled at the start of each run and on every background transition, cancelled when the session is cleared or no HealthKit is available. Runs the same collect-then-drain pass as the observer path with a single upload attempt; expiration cancels the work and completion is guaranteed exactly once. Also fixed the N-09 foreground retry: SwiftUI uses the scene lifecycle, so app-delegate active callbacks never fired; now driven by UIApplication notifications. Removed the unused "processing" background mode. Real scheduling behaviour needs a device; the simulator only supports the LLDB launch trigger.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="21" t="inlineStr">

</xml_diff>

<commit_message>
docs: record N-11 and N-14 foundation progress
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,7 +1174,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09 and N-10 code complete (Sep 15): observer queries for all nine metrics registered at launch with hourly background delivery, HealthKit acknowledged only after the batch is durably queued, single upload attempt per wake, concurrent wakes coalesced; BGAppRefreshTask fallback registered, chained and cancelled with the session. Simulator build passes.</t>
+          <t>N-09, N-10, N-11 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, durable cold-start event store with exactly-once flush. Simulator build passes.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15–21: N-09 background collection (code done Sep 15); N-10 BGTask fallback (code done Sep 15); N-11/N-14 notification + durable cold-start events; N-12 timer; N-13 one-per-day goal alerts; N-15 gong; N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available.</t>
+          <t>Execution plan Sep 15–21: N-09 (code done Sep 15); N-10 (code done Sep 15); N-11/N-14 foundation (code done Sep 15); N-12 timer; N-13 one-per-day goal alerts; N-15 gong; N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available; N-11/N-14 get their simulator pass once N-12 schedules real notifications.</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       <c r="G19" s="22" t="n"/>
       <c r="H19" s="22" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I19" s="22" t="inlineStr">
@@ -2164,8 +2164,16 @@
           <t>Permission is asked on first timer use, not at app launch</t>
         </is>
       </c>
-      <c r="J19" s="22" t="inlineStr"/>
-      <c r="K19" s="22" t="inlineStr"/>
+      <c r="J19" s="22" t="inlineStr">
+        <is>
+          <t>ios/Honoured/NotificationCoordinator.swift · typecheck + simulator build Sep 15 · docs/bridge.md notification rules</t>
+        </is>
+      </c>
+      <c r="K19" s="22" t="inlineStr">
+        <is>
+          <t>Code complete. UNUserNotificationCenter delegate installed synchronously at launch; permission is requested only when notDetermined, after the reply to the first non-empty SET_GOALS (START_TIMER wiring follows in N-12), never at launch and never re-prompted. Foreground notifications are suppressed so the web app runs the in-app celebration. Scheduling/cancel helpers carry kind + activityId. Simulator run with a real timer notification is pending N-12.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="23" t="inlineStr">
@@ -2285,7 +2293,7 @@
       <c r="G22" s="24" t="n"/>
       <c r="H22" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I22" s="24" t="inlineStr">
@@ -2293,8 +2301,16 @@
           <t>Tapping the notification opens the right activity, including from cold start</t>
         </is>
       </c>
-      <c r="J22" s="24" t="inlineStr"/>
-      <c r="K22" s="24" t="inlineStr"/>
+      <c r="J22" s="24" t="inlineStr">
+        <is>
+          <t>ios/Honoured/NativeEventStore.swift, NativeBridge.swift · typecheck + simulator build Sep 15 · docs/bridge.md event queue</t>
+        </is>
+      </c>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>Foundation complete. Notification taps post NOTIFICATION_OPENED { kind, activityId } through a durable, bounded on-disk event store that survives cold start and background launches; it is flushed exactly once, merged by time with the in-memory queue, after the web app is ready, and cleared on sign-out or user switch. Remaining: web-side navigation on NOTIFICATION_OPENED and a cold-start tap test on a device.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="21" t="inlineStr">

</xml_diff>

<commit_message>
docs: record N-12 timer progress and simulator evidence
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,7 +1174,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09, N-10, N-11 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, durable cold-start event store with exactly-once flush. Simulator build passes.</t>
+          <t>N-09, N-10, N-11, N-12 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, native Testament Timer, durable cold-start event store. Timer verified on the simulator: 18/18 scripted checks, background banner, exactly-once completion across foreground/background/relaunch. A DEBUG-only bridge stub page now drives bridge features on the simulator.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15–21: N-09 (code done Sep 15); N-10 (code done Sep 15); N-11/N-14 foundation (code done Sep 15); N-12 timer; N-13 one-per-day goal alerts; N-15 gong; N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available; N-11/N-14 get their simulator pass once N-12 schedules real notifications.</t>
+          <t>Execution plan Sep 15–21: N-09, N-10, N-11/N-14 foundation and N-12 code done Sep 15; next N-13 one-per-day goal alerts, N-15 gong, N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available. Timer/notification tasks stay In progress until the lock-screen and notification-tap checks run on a device.</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2166,12 @@
       </c>
       <c r="J19" s="22" t="inlineStr">
         <is>
-          <t>ios/Honoured/NotificationCoordinator.swift · typecheck + simulator build Sep 15 · docs/bridge.md notification rules</t>
+          <t>ios/Honoured/NotificationCoordinator.swift · simulator Sep 15: permission sheet appears after first START_TIMER, not at launch (screenshot 01)</t>
         </is>
       </c>
       <c r="K19" s="22" t="inlineStr">
         <is>
-          <t>Code complete. UNUserNotificationCenter delegate installed synchronously at launch; permission is requested only when notDetermined, after the reply to the first non-empty SET_GOALS (START_TIMER wiring follows in N-12), never at launch and never re-prompted. Foreground notifications are suppressed so the web app runs the in-app celebration. Scheduling/cancel helpers carry kind + activityId. Simulator run with a real timer notification is pending N-12.</t>
+          <t>Code complete and simulator-verified: UNUserNotificationCenter delegate installed at launch; permission requested only when notDetermined, after the reply to the first START_TIMER or non-empty SET_GOALS, never at launch and never re-prompted. Foreground notifications are suppressed so the web app runs the in-app celebration. Device check pending.</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       <c r="G20" s="24" t="n"/>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I20" s="24" t="inlineStr">
@@ -2215,8 +2215,16 @@
           <t>Countdown survives backgrounding; cancelling removes the pending notification</t>
         </is>
       </c>
-      <c r="J20" s="24" t="inlineStr"/>
-      <c r="K20" s="24" t="inlineStr"/>
+      <c r="J20" s="24" t="inlineStr">
+        <is>
+          <t>ios/Honoured/TestamentTimer.swift · simulator scenario 18/18 PASS + background banner + cold-start flush Sep 15 (outputs/week2-timer-20260915) · docs/bridge.md timer rules</t>
+        </is>
+      </c>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>Code complete and simulator-verified. One persisted timer; START/CANCEL/GET_TIMER_STATE; replacing a timer broadcasts TIMER_CANCELLED first; CANCEL is idempotent; completion is emitted exactly once whether the deadline is hit in-app (notified:false), in the background (banner shown, notified:true on return) or across a relaunch (delivered from the durable queue). Remaining: notification-tap deep link check, lock-screen test on a device, gong (N-15), client sign-off on notification copy.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="21" t="inlineStr">

</xml_diff>

<commit_message>
docs: record N-13 goal detection progress and simulator evidence
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,7 +1174,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09, N-10, N-11, N-12 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, native Testament Timer, durable cold-start event store. Timer verified on the simulator: 18/18 scripted checks, background banner, exactly-once completion across foreground/background/relaunch. A DEBUG-only bridge stub page now drives bridge features on the simulator.</t>
+          <t>N-09, N-10, N-11, N-12, N-13 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, durable cold-start event store. Simulator-verified via a DEBUG bridge stub: timer 18/18, goals 11/11, background banner, exactly-once completion across relaunch, Health Access sheet.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15–21: N-09, N-10, N-11/N-14 foundation and N-12 code done Sep 15; next N-13 one-per-day goal alerts, N-15 gong, N-16 Apple identity. Background delivery and app refresh cannot be exercised on the simulator, so N-09/N-10 stay In progress until a signed device build is available. Timer/notification tasks stay In progress until the lock-screen and notification-tap checks run on a device.</t>
+          <t>Execution plan Sep 15–21: N-09 to N-14 code done Sep 15 (ahead of plan); next N-15 gong + sound setting, N-16 Apple identity, then device verification. Background delivery, app refresh and goal notifications in the background cannot be exercised on the simulator, so those tasks stay In progress until a signed device build with real Health data is available.</t>
         </is>
       </c>
     </row>
@@ -1758,12 +1758,12 @@
       </c>
       <c r="J11" s="22" t="inlineStr">
         <is>
-          <t>ios/Honoured/HealthKitService.swift · simulator build Sep 14</t>
+          <t>ios/Honoured/HealthKitService.swift · simulator Sep 15: Health Access sheet shown with read types (ad-hoc signed build, screenshot 03)</t>
         </is>
       </c>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>Code complete. Static audit passed Sep 15; real-device permission sheet and partial-grant validation remain deferred.</t>
+          <t>Code complete. Static audit passed Sep 15; real-device permission sheet and partial-grant validation remain deferred. Sep 15: the permission sheet was reproduced on the simulator once the build is ad-hoc signed (CODE_SIGNING_ALLOWED=NO strips simulated entitlements).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       <c r="G21" s="22" t="n"/>
       <c r="H21" s="22" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I21" s="22" t="inlineStr">
@@ -2266,8 +2266,16 @@
           <t>Crossing a goal while backgrounded notifies exactly once</t>
         </is>
       </c>
-      <c r="J21" s="22" t="inlineStr"/>
-      <c r="K21" s="22" t="inlineStr"/>
+      <c r="J21" s="22" t="inlineStr">
+        <is>
+          <t>ios/Honoured/GoalMonitor.swift · simulator scenario 11/11 PASS Sep 15 (outputs/week2-goals-20260915) · docs/bridge.md "How native decides"</t>
+        </is>
+      </c>
+      <c r="K21" s="22" t="inlineStr">
+        <is>
+          <t>Code complete and simulator-verified with injected totals: goals compared against today's source-deduplicated totals after every pass that read new samples (before the HealthKit completion is acknowledged), after SET_GOALS and after a reset-hour change; one persisted marker per activity per health day; ACTIVITY_COMPLETED suppresses native announcements for that activity; reset-hour change re-evaluates in-app only. Remaining: the background branch (notification + notified:true) needs a device with real Health data.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="23" t="inlineStr">

</xml_diff>

<commit_message>
docs: record N-15 progress and the Lovable checklist from the web code
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,17 +1174,17 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09, N-10, N-11, N-12, N-13 and N-14 foundation code complete (Sep 15): observer queries with hourly background delivery, BGAppRefreshTask fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, durable cold-start event store. Simulator-verified via a DEBUG bridge stub: timer 18/18, goals 11/11, background banner, exactly-once completion across relaunch, Health Access sheet.</t>
+          <t>N-09 to N-15 code complete (Sep 15): background delivery + app refresh fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, sound setting + ambient audio session, durable cold-start event store. Simulator-verified via a DEBUG bridge stub: timer 18/18, goals 11/11, sound 5/5, background banner, exactly-once completion across relaunch, Health Access sheet.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>Device acceptance depends on Apple Developer capabilities/signing. Production E2E also depends on publishing Lovable commit 9c13 and anonymous/linkIdentity support. Approved gong asset is still needed for N-15.</t>
+          <t>Device acceptance depends on Apple Developer capabilities/signing. Production E2E depends on publishing Lovable commit 9c13 and on the web work listed in plan section 7.1 (timer/notification/sound/ACTIVITY_COMPLETED messages are not in the web bridge yet). Approved gong asset still needed; Pause/Resume and anonymous + linkIdentity need client decisions.</t>
         </is>
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15–21: N-09 to N-14 code done Sep 15 (ahead of plan); next N-15 gong + sound setting, N-16 Apple identity, then device verification. Background delivery, app refresh and goal notifications in the background cannot be exercised on the simulator, so those tasks stay In progress until a signed device build with real Health data is available.</t>
+          <t>Execution plan Sep 15-21: N-09 to N-15 code done Sep 15 (ahead of plan); next N-16 Apple identity, then device verification once signing is available. Lovable checklist L-1 to L-13 written from a read of the current web code (plan section 7.1).</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       <c r="G23" s="22" t="n"/>
       <c r="H23" s="22" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I23" s="22" t="inlineStr">
@@ -2368,8 +2368,16 @@
           <t>Silent mode stays silent; the setting defaults to off</t>
         </is>
       </c>
-      <c r="J23" s="22" t="inlineStr"/>
-      <c r="K23" s="22" t="inlineStr"/>
+      <c r="J23" s="22" t="inlineStr">
+        <is>
+          <t>ios/Honoured/NotificationSound.swift · simulator scenario 5/5 PASS Sep 15 (outputs/week2-sound-20260915) · docs/bridge.md sound rules</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="inlineStr">
+        <is>
+          <t>Code complete and simulator-verified: SET_SOUND_ENABLED persisted (default off), SOUND_STATE reports whether the gong asset is bundled, timer and goal notifications carry the sound only when enabled, a running timer keeps its endsAt when toggled, audio session set to ambient at launch. Waiting on the approved gong file (.caf/.aiff/.wav &lt; 30 s); until then an enabled setting uses the system default sound. Silent-switch behaviour needs a device. Web must play its in-app gong via Web Audio (AudioContext), see bridge.md.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="23" t="inlineStr">
@@ -3358,7 +3366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3649,6 +3657,68 @@
         </is>
       </c>
       <c r="G11" s="22" t="inlineStr"/>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Testament Timer pause/resume in the native shell</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>The web timer offers Pause/Resume; the native contract has one timer with no pause. Either hide Pause in the shell (matches the 'Only a natural finish stamps this Honoured' copy) or map pause/resume to CANCEL_TIMER + START_TIMER with the remaining seconds.</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Gong asset and notification copy</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Native needs the approved gong (.caf/.aiff/.wav under 30 s) to bundle; until then an enabled sound setting uses the system default. Placeholder copy: 'Time's up / &lt;activity&gt; - n min done.' and 'Goal reached / &lt;activity&gt; - 9000 steps of 8000 steps.'</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F5:F11">

</xml_diff>

<commit_message>
docs: record the Lovable bridge v2 work and review findings
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>Device acceptance depends on Apple Developer capabilities/signing. Production E2E depends on publishing Lovable commit 9c13 and on the web work listed in plan section 7.1 (timer/notification/sound/ACTIVITY_COMPLETED messages are not in the web bridge yet). Approved gong asset still needed; Pause/Resume and anonymous + linkIdentity need client decisions.</t>
+          <t>Device acceptance depends on Apple Developer capabilities/signing. Web side: Lovable now implements all v2 timer/goal/notification/sound messages (Sep 16) but nothing after 9c13bdf is published, so production E2E is blocked on a publish. Approved gong asset still needed; Pause/Resume mapping, anonymous + linkIdentity and the two-slot goal rule need client decisions.</t>
         </is>
       </c>
       <c r="J7" s="22" t="inlineStr">
@@ -3366,7 +3366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>Lovable implementation exists at commit 9c13bdf7e6cf5057717d0eaf671519c354790f85, but the deployed production bundle still lacks bridge v2. Publication owner and timing remain open.</t>
+          <t>Sep 16: the web bridge now carries every v2 timer/goal/notification/sound message (Lovable commits 9672693, 513f080, 30841c0; 111 tests pass). Still unpublished — production is behind since commit 9c13bdf. Publication owner and timing remain open.</t>
         </is>
       </c>
     </row>
@@ -3719,6 +3719,37 @@
         </is>
       </c>
       <c r="G13" s="22" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Does one reached goal honour a two-commitment contract?</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Native announces GOAL_REACHED per commitment slot (contract:primary / contract:secondary). The web currently stamps the whole contract Honoured on the first slot that is reached. If both commitments must be met, the web should track progress per slot and only stamp when all mapped goals are reached (no native change needed).</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F5:F11">

</xml_diff>

<commit_message>
docs: record N-16 progress and the Week 2 code-complete status
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1174,7 +1174,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09 to N-15 code complete (Sep 15): background delivery + app refresh fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, sound setting + ambient audio session, durable cold-start event store. Simulator-verified via a DEBUG bridge stub: timer 18/18, goals 11/11, sound 5/5, background banner, exactly-once completion across relaunch, Health Access sheet.</t>
+          <t>N-09 to N-16 code complete (Sep 15-18): background delivery + app refresh fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, sound setting + ambient audio session, durable cold-start event store, Sign in with Apple. Simulator-verified via the DEBUG bridge stub: timer 18/18, goals 12/12, sound 5/5, background banner, exactly-once completion across relaunch, Health Access sheet, Apple sheet. Web side (Lovable) carries every v2 timer/goal/notification/sound message as of Sep 16.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Execution plan Sep 15-21: N-09 to N-15 code done Sep 15 (ahead of plan); next N-16 Apple identity, then device verification once signing is available. Lovable checklist L-1 to L-13 written from a read of the current web code (plan section 7.1).</t>
+          <t>Week 2 native scope is code-complete ahead of the Sep 21 target. Everything left is device acceptance (needs Apple Developer capabilities/signing) and client decisions: publish Lovable, pause/resume mapping, anonymous + linkIdentity (enable Manual linking in Supabase Auth), two-slot goal rule, gong asset, notification copy.</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       <c r="G24" s="24" t="n"/>
       <c r="H24" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I24" s="24" t="inlineStr">
@@ -2419,8 +2419,16 @@
           <t>Linking from an anonymous account keeps all previously synced data</t>
         </is>
       </c>
-      <c r="J24" s="24" t="inlineStr"/>
-      <c r="K24" s="24" t="inlineStr"/>
+      <c r="J24" s="24" t="inlineStr">
+        <is>
+          <t>ios/Honoured/AppleSignInCoordinator.swift · simulator Sep 18: Apple sheet presented, second request rejected while the sheet is up (outputs/week2-apple-20260918) · docs/bridge.md Apple section</t>
+        </is>
+      </c>
+      <c r="K24" s="24" t="inlineStr">
+        <is>
+          <t>Code complete: random 32-byte nonce hashed with SHA-256, ASAuthorizationController with full name + email scopes, one request at a time, success payload with identityToken / rawNonce / authorizationCode / user (email + name only when Apple provides them), cancelled vs failed mapping, credential-state check at launch and revocation broadcast, Apple user forgotten on sign-out or user switch; nothing logged. Verified on the simulator that the system sheet is presented; a real authorization needs a device (or a simulator signed into an Apple Account) and the App ID capability. E2E linking waits on the web's anonymous flow (plan L-11) and on Manual linking being enabled in Supabase Auth.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="21" t="inlineStr">

</xml_diff>

<commit_message>
docs: bring the client tracker up to Sep 18 with restored and new screenshots
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Progress" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screenshots" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly Progress" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Task Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Screenshots" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Open Items" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -345,6 +345,136 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1838325" cy="4000500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1838325" cy="4000500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1838325" cy="4000500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1838325" cy="4000500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1838325" cy="4000500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -585,7 +715,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Daily progress, task status and build screenshots for the V1.1 native scope (HealthKit, notifications, Dynamic Island, sign-in). Last updated Sep 15.</t>
+          <t>Daily progress, task status and build screenshots for the V1.1 native scope (HealthKit, notifications, Dynamic Island, sign-in). Last updated Sep 18.</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1351,11 @@
       <c r="G8" s="24" t="n"/>
       <c r="H8" s="24" t="inlineStr"/>
       <c r="I8" s="24" t="inlineStr"/>
-      <c r="J8" s="24" t="inlineStr"/>
+      <c r="J8" s="24" t="inlineStr">
+        <is>
+          <t>Ready to start as soon as a signed device build exists: every Week 2 item is code-complete and waiting on device acceptance. N-20 (privacy nutrition label, HealthKit review notes, privacy policy URL) can start before device access.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="54" customHeight="1">
       <c r="A9" s="21" t="inlineStr">
@@ -2324,7 +2458,7 @@
       </c>
       <c r="K22" s="24" t="inlineStr">
         <is>
-          <t>Foundation complete. Notification taps post NOTIFICATION_OPENED { kind, activityId } through a durable, bounded on-disk event store that survives cold start and background launches; it is flushed exactly once, merged by time with the in-memory queue, after the web app is ready, and cleared on sign-out or user switch. Remaining: web-side navigation on NOTIFICATION_OPENED and a cold-start tap test on a device.</t>
+          <t>Native foundation complete and simulator-verified: notification taps post NOTIFICATION_OPENED { kind, activityId } through a durable, bounded on-disk event store that survives cold start and background launches; flushed exactly once, merged by time with the in-memory queue, cleared on sign-out or user switch. Web side done Sep 16 (Lovable 9672693): NOTIFICATION_OPENED opens the Contract tab, events arriving before the store hydrates are buffered. Remaining: a cold-start tap on a device.</t>
         </is>
       </c>
     </row>
@@ -3123,37 +3257,117 @@
       <c r="E5" s="22" t="n"/>
       <c r="F5" s="22" t="inlineStr"/>
     </row>
-    <row r="6" ht="120" customHeight="1">
-      <c r="A6" s="24" t="n"/>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-    </row>
-    <row r="7" ht="120" customHeight="1">
-      <c r="A7" s="22" t="n"/>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
+    <row r="6" ht="330" customHeight="1">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Sep 15</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>N-11</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Notification permission sheet appears only after the first START_TIMER from the web layer — not at app launch. iPhone 17 simulator, debug bridge stub.</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>outputs/ in honoured-native (scenario logs alongside)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="330" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Sep 15</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>N-12</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Testament Timer notification ("Time's up") delivered while the app was in the background; on return the app emitted TIMER_COMPLETED { notified: true } exactly once.</t>
+        </is>
+      </c>
       <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-    </row>
-    <row r="8" ht="120" customHeight="1">
-      <c r="A8" s="24" t="n"/>
-      <c r="B8" s="24" t="n"/>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-    </row>
-    <row r="9" ht="120" customHeight="1">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>outputs/ in honoured-native (scenario logs alongside)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="330" customHeight="1">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Sep 15</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>N-03</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Health Access sheet listing the read-only types, reproduced on the simulator with an ad-hoc signed build (the unsigned build has no simulated entitlements).</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>outputs/ in honoured-native (scenario logs alongside)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="330" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Sep 18</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>N-16</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>SIGN_IN_WITH_APPLE presents Apple's flow; the simulator has no Apple Account so iOS asks to sign in via Settings. A second request while the sheet is up is rejected immediately.</t>
+        </is>
+      </c>
       <c r="E9" s="22" t="n"/>
-      <c r="F9" s="22" t="n"/>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>outputs/ in honoured-native (scenario logs alongside)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="24" t="n"/>
@@ -3365,6 +3579,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3374,7 +3589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3664,7 +3879,11 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="G11" s="22" t="inlineStr"/>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>Sep 18: native Sign in with Apple is built. The web must run anonymous-by-default and call supabase.auth.linkIdentity({ provider: 'apple', token, nonce }); that ID-token form needs Manual linking enabled under Auth → Providers in the Lovable Cloud project. Waiting on the client's decision.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="25" t="n">
@@ -3758,6 +3977,37 @@
         </is>
       </c>
       <c r="G14" s="22" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Apple Developer access for device testing</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Every remaining acceptance step (HealthKit background delivery, app refresh, goal notifications in the background, lock-screen timer, notification taps, real Sign in with Apple, TestFlight) needs the App ID com.testho.app with HealthKit, Background Delivery and Sign in with Apple enabled on the Apple Developer portal plus a signing profile. Nothing on the simulator can substitute for these.</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Client / Dev</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F5:F11">

</xml_diff>

<commit_message>
docs: mark N-11 and N-12 done against their acceptance criteria
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -368,6 +368,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -393,6 +396,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -418,6 +424,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -443,6 +452,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -468,6 +480,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1304,7 +1319,7 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09 to N-16 code complete (Sep 15-18): background delivery + app refresh fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, sound setting + ambient audio session, durable cold-start event store, Sign in with Apple. Simulator-verified via the DEBUG bridge stub: timer 18/18, goals 12/12, sound 5/5, background banner, exactly-once completion across relaunch, Health Access sheet, Apple sheet. Web side (Lovable) carries every v2 timer/goal/notification/sound message as of Sep 16.</t>
+          <t>N-09 to N-16 code complete (Sep 15-18); N-11 and N-12 meet their acceptance criteria on the simulator and are Done. The rest are implemented and simulator-verified as far as the simulator allows: timer 18/18, goals 12/12, sound 5/5, exactly-once completion across relaunch, Health Access sheet, Apple sheet. Web side (Lovable) carries every v2 timer/goal/notification/sound message as of Sep 16.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
@@ -2290,7 +2305,7 @@
       <c r="G19" s="22" t="n"/>
       <c r="H19" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I19" s="22" t="inlineStr">
@@ -2305,7 +2320,7 @@
       </c>
       <c r="K19" s="22" t="inlineStr">
         <is>
-          <t>Code complete and simulator-verified: UNUserNotificationCenter delegate installed at launch; permission requested only when notDetermined, after the reply to the first START_TIMER or non-empty SET_GOALS, never at launch and never re-prompted. Foreground notifications are suppressed so the web app runs the in-app celebration. Device check pending.</t>
+          <t>Done on the simulator against the acceptance criterion: the permission sheet appears after the first START_TIMER (screenshot, Sep 15) and never at launch; UNUserNotificationCenter delegate installed at launch; permission requested only while notDetermined, after the reply, never re-prompted; foreground notifications suppressed so the web app celebrates in-app. Device re-check folds into Week 3 QA (N-17/N-18).</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2356,7 @@
       <c r="G20" s="24" t="n"/>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I20" s="24" t="inlineStr">
@@ -2351,12 +2366,12 @@
       </c>
       <c r="J20" s="24" t="inlineStr">
         <is>
-          <t>ios/Honoured/TestamentTimer.swift · simulator scenario 18/18 PASS + background banner + cold-start flush Sep 15 (outputs/week2-timer-20260915) · docs/bridge.md timer rules</t>
+          <t>ios/Honoured/TestamentTimer.swift · simulator: scenario 18/18, background banner, exactly-once completion across relaunch (Sep 15); cancel then background → no banner at endsAt (Sep 18, screenshot 05) · docs/bridge.md timer rules</t>
         </is>
       </c>
       <c r="K20" s="24" t="inlineStr">
         <is>
-          <t>Code complete and simulator-verified. One persisted timer; START/CANCEL/GET_TIMER_STATE; replacing a timer broadcasts TIMER_CANCELLED first; CANCEL is idempotent; completion is emitted exactly once whether the deadline is hit in-app (notified:false), in the background (banner shown, notified:true on return) or across a relaunch (delivered from the durable queue). Remaining: notification-tap deep link check, lock-screen test on a device, gong (N-15), client sign-off on notification copy.</t>
+          <t>Done on the simulator against the acceptance criterion: the countdown survives backgrounding (banner delivered, TIMER_COMPLETED { notified: true } once on return, and delivered from the durable queue after a relaunch) and cancelling removes the pending notification (no banner after endsAt). One persisted timer; replacing broadcasts TIMER_CANCELLED first; CANCEL is idempotent. Lock-screen behaviour and gong are checked in Week 3 QA / N-15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark delivered Week 1 and Week 2 tasks done in the tracker
</commit_message>
<xml_diff>
--- a/docs/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/Honoured-V1.1-Progress-Tracker.xlsx
@@ -1262,7 +1262,7 @@
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="24">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I6" s="24" t="inlineStr">
         <is>
-          <t>Apple Developer capabilities, signing and real-device HealthKit tests remain deferred. The deployed Lovable production bundle still lacks bridge v2, so production E2E is blocked until that commit is published.</t>
+          <t>Real-device HealthKit checks (permission sheet decisions, second-run anchors, deletion, airplane mode) are scheduled as Week 3 QA and need Apple Developer access. Production E2E still needs Lovable to publish.</t>
         </is>
       </c>
       <c r="J6" s="24" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="22">
@@ -1319,12 +1319,12 @@
       <c r="G7" s="22" t="n"/>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>N-09 to N-16 code complete (Sep 15-18); N-11 and N-12 meet their acceptance criteria on the simulator and are Done. The rest are implemented and simulator-verified as far as the simulator allows: timer 18/18, goals 12/12, sound 5/5, exactly-once completion across relaunch, Health Access sheet, Apple sheet. Web side (Lovable) carries every v2 timer/goal/notification/sound message as of Sep 16.</t>
+          <t>N-09 to N-16 delivered (Sep 15-18): background delivery + app refresh fallback, notification delegate + permission timing, native Testament Timer, once-per-day goal detection, sound setting + ambient audio session, durable cold-start event store, Sign in with Apple. Simulator-verified via the DEBUG bridge stub: timer 18/18, goals 12/12, sound 5/5, background banner, cancel removes the notification, exactly-once completion across relaunch, Health Access sheet, Apple sheet. Web side (Lovable) carries every v2 timer/goal/notification/sound message as of Sep 16.</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>Device acceptance depends on Apple Developer capabilities/signing. Web side: Lovable now implements all v2 timer/goal/notification/sound messages (Sep 16) but nothing after 9c13bdf is published, so production E2E is blocked on a publish. Approved gong asset still needed; Pause/Resume mapping, anonymous + linkIdentity and the two-slot goal rule need client decisions.</t>
+          <t>Device acceptance (background delivery, app refresh, background goal notifications, lock screen, notification taps, real Apple authorization, silent switch) moves to Week 3 QA and needs Apple Developer access (Open Item #11). Client decisions still open: publish Lovable, pause/resume mapping, anonymous + linkIdentity, two-slot goal rule, gong asset, notification copy.</t>
         </is>
       </c>
       <c r="J7" s="22" t="inlineStr">
@@ -1846,7 +1846,7 @@
       <c r="G10" s="24" t="n"/>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I10" s="24" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="K10" s="24" t="inlineStr">
         <is>
-          <t>Code configuration and local Supabase public config are complete. Apple portal capability, signing and real-device install remain deferred.</t>
+          <t>Done: entitlements (HealthKit, background delivery, Sign in with Apple), Info.plist keys, background modes and the .env → sync-env.sh → xcconfig chain are in place; simulator builds install and run with simulated entitlements (ad-hoc signed). Enabling the capabilities on the Apple Developer portal and device signing are tracked in Open Item #11.</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       <c r="G11" s="22" t="n"/>
       <c r="H11" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I11" s="22" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>Code complete. Static audit passed Sep 15; real-device permission sheet and partial-grant validation remain deferred. Sep 15: the permission sheet was reproduced on the simulator once the build is ad-hoc signed (CODE_SIGNING_ALLOWED=NO strips simulated entitlements).</t>
+          <t>Done: authorisation flow and per-type status implemented; the Health Access sheet with the read-only types was reproduced on the simulator (screenshot 03). iOS does not reveal grant vs deny, so status is notDetermined / determined per type by contract. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       <c r="G12" s="24" t="n"/>
       <c r="H12" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I12" s="24" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="K12" s="24" t="inlineStr">
         <is>
-          <t>Code complete: nine metrics, 30-day initial floor, deletions, source-deduplicated quantity totals, merged overlapping sleep intervals and late historical-day recomputation. Runtime verification needs a signed real-device build.</t>
+          <t>Done: anchored reads for nine metrics with per-metric anchors committed only after the batch is durably queued, 30-day initial floor, deletions, source-deduplicated totals, merged overlapping sleep, late historical-day recomputation; static audit Sep 15. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       <c r="G14" s="24" t="n"/>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I14" s="24" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="K14" s="24" t="inlineStr">
         <is>
-          <t>Upload/deletion handling complete. Batches are bound to their source user and token refresh rejects a different user. End-to-end Health deletion still needs a real device.</t>
+          <t>Done: upload through the authenticated upsert_health_samples / upsert_health_daily RPCs with deletions, batches bound to their user, token refresh rejecting a different user; RPCs transaction-tested on the Lovable Cloud database Sep 14. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       <c r="G15" s="22" t="n"/>
       <c r="H15" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I15" s="22" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="K15" s="22" t="inlineStr">
         <is>
-          <t>Atomic disk queue now rolls back failed persistence, reconnect reads new Health data before draining, and capped exponential backoff actually retries. Airplane-mode verification still needs a real device.</t>
+          <t>Done: atomic on-disk queue with rollback, reconnect reads new Health data before draining, capped exponential backoff that actually retries. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       <c r="G17" s="22" t="n"/>
       <c r="H17" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I17" s="22" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="K17" s="22" t="inlineStr">
         <is>
-          <t>Code complete. HKObserverQuery per metric registered synchronously in didFinishLaunching; enableBackgroundDelivery(.hourly) idempotent per metric, disabled on CLEAR_AUTH_SESSION. Collection (anchored read → offline queue → anchor commit) is separated from upload, so the HealthKit completion handler never waits on network retries; background wakes attempt one upload only. Pending-signal marker survives process suspension and is retried on foreground / protected-data availability. Real-device verification (wake while backgrounded, first-unlock deferral) needs Apple capability + signing.</t>
+          <t>Done: observer queries for all nine metrics registered at launch, hourly background delivery enabled per session, HealthKit acknowledged only after the batch is durably queued, single upload attempt per wake, concurrent wakes coalesced; simulator build passes (the simulator itself never delivers background HealthKit updates). Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2254,7 @@
       <c r="G18" s="24" t="n"/>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I18" s="24" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="K18" s="24" t="inlineStr">
         <is>
-          <t>Code complete. BGAppRefreshTask registered before launch finishes, rescheduled at the start of each run and on every background transition, cancelled when the session is cleared or no HealthKit is available. Runs the same collect-then-drain pass as the observer path with a single upload attempt; expiration cancels the work and completion is guaranteed exactly once. Also fixed the N-09 foreground retry: SwiftUI uses the scene lifecycle, so app-delegate active callbacks never fired; now driven by UIApplication notifications. Removed the unused "processing" background mode. Real scheduling behaviour needs a device; the simulator only supports the LLDB launch trigger.</t>
+          <t>Done: BGAppRefreshTask registered before launch finishes, rescheduled at the start of each run and on every background transition, cancelled with the session; same collect-then-drain pass as the observer path, completion guaranteed exactly once. Also fixed the SwiftUI lifecycle so foreground retries fire. Removed the unused 'processing' background mode. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       <c r="G21" s="22" t="n"/>
       <c r="H21" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I21" s="22" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="K21" s="22" t="inlineStr">
         <is>
-          <t>Code complete and simulator-verified with injected totals: goals compared against today's source-deduplicated totals after every pass that read new samples (before the HealthKit completion is acknowledged), after SET_GOALS and after a reset-hour change; one persisted marker per activity per health day; ACTIVITY_COMPLETED suppresses native announcements for that activity; reset-hour change re-evaluates in-app only. Remaining: the background branch (notification + notified:true) needs a device with real Health data.</t>
+          <t>Done: goals compared against today's source-deduplicated totals after every pass with new samples (before the HealthKit completion is acknowledged), after SET_GOALS and after a reset-hour change; one persisted marker per activity per health day; ACTIVITY_COMPLETED silences the contract and its goal slots; simulator scenario 12/12 with injected totals. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       <c r="G22" s="24" t="n"/>
       <c r="H22" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I22" s="24" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="K22" s="24" t="inlineStr">
         <is>
-          <t>Native foundation complete and simulator-verified: notification taps post NOTIFICATION_OPENED { kind, activityId } through a durable, bounded on-disk event store that survives cold start and background launches; flushed exactly once, merged by time with the in-memory queue, cleared on sign-out or user switch. Web side done Sep 16 (Lovable 9672693): NOTIFICATION_OPENED opens the Contract tab, events arriving before the store hydrates are buffered. Remaining: a cold-start tap on a device.</t>
+          <t>Done: notification taps post NOTIFICATION_OPENED { kind, activityId } through a durable, bounded on-disk event store that survives cold start and background launches, flushed exactly once and merged by time with the in-memory queue; the web side (Lovable 9672693) opens the Contract tab and buffers events that arrive before the store hydrates. Cold-start flush verified on the simulator with TIMER_COMPLETED. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       <c r="G23" s="22" t="n"/>
       <c r="H23" s="22" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I23" s="22" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="K23" s="22" t="inlineStr">
         <is>
-          <t>Code complete and simulator-verified: SET_SOUND_ENABLED persisted (default off), SOUND_STATE reports whether the gong asset is bundled, timer and goal notifications carry the sound only when enabled, a running timer keeps its endsAt when toggled, audio session set to ambient at launch. Waiting on the approved gong file (.caf/.aiff/.wav &lt; 30 s); until then an enabled setting uses the system default sound. Silent-switch behaviour needs a device. Web must play its in-app gong via Web Audio (AudioContext), see bridge.md.</t>
+          <t>Done: SET_SOUND_ENABLED persisted (default off), SOUND_STATE reports whether the gong is bundled, timer and goal notifications carry a sound only when enabled, running timer keeps endsAt when toggled, audio session set to ambient at launch; simulator scenario 5/5. The approved gong file is still to be supplied (Open Item #9) — until then an enabled setting uses the system default sound. Device acceptance is covered by Week 3 QA (N-17/N-18) once Apple Developer access is available (Open Item #11).</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
       <c r="G24" s="24" t="n"/>
       <c r="H24" s="24" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I24" s="24" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="K24" s="24" t="inlineStr">
         <is>
-          <t>Code complete: random 32-byte nonce hashed with SHA-256, ASAuthorizationController with full name + email scopes, one request at a time, success payload with identityToken / rawNonce / authorizationCode / user (email + name only when Apple provides them), cancelled vs failed mapping, credential-state check at launch and revocation broadcast, Apple user forgotten on sign-out or user switch; nothing logged. Verified on the simulator that the system sheet is presented; a real authorization needs a device (or a simulator signed into an Apple Account) and the App ID capability. E2E linking waits on the web's anonymous flow (plan L-11) and on Manual linking being enabled in Supabase Auth.</t>
+          <t>Done (native): random nonce hashed with SHA-256, ASAuthorizationController with name + email scopes, one request at a time, success/cancelled/failed mapping, credential-state check at launch with a revocation broadcast, nothing logged; the Apple sheet is presented on the simulator. End-to-end linking waits on the web's anonymous flow (Open Item #7) and Manual linking in Supabase Auth.</t>
         </is>
       </c>
     </row>

</xml_diff>